<commit_message>
feat(table): FlappyConfig에 대시 튜닝값 4열
dash_mult 2 / dash_duration 0.2 / dash_charge_base 0.13 / dash_charge_dive 1.2.
값은 옛 싱글 프로토타입(FlappyPlayer)에서 그대로 가져왔다.

충전량을 "기본 + 낙하 비례"로 두 열로 나눈 이유는 그 둘이 서로 다른 것을 조절하기
때문이다 — 기본은 가만히 있어도 차는 최소 속도(대시를 아예 못 쓰는 구간을 막는다),
낙하 몫은 위험을 감수한 보상의 크기다. 한 값으로 합치면 둘 중 하나만 만지고 싶을 때
반드시 다른 하나가 딸려 움직인다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SUnLXZFg9TeqE7mgvUt1Vp
</commit_message>
<xml_diff>
--- a/table/Datas/#FlappyConfig.xlsx
+++ b/table/Datas/#FlappyConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,26 @@
           <t>invuln_time</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dash_mult</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>dash_duration</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>dash_charge_base</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>dash_charge_dive</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -529,6 +549,26 @@
           <t>float</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -591,6 +631,26 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>invuln_time</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>dash_mult</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>dash_duration</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>dash_charge_base</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>dash_charge_dive</t>
         </is>
       </c>
     </row>
@@ -624,6 +684,18 @@
       </c>
       <c r="K5" t="n">
         <v>0.6</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(table): 추격자 곡선 값 네 개를 FlappyConfig에 넣는다
시작점 -60, 초기속도 7, 가속 0.075, 상한 10. 프로토타입에서 튜닝해 둔 값을
그대로 옮긴다 — 코스가 632m로 같아서 그대로 성립한다.

상한 10이 전진속도 11보다 낮은 것이 핵심이다. 이것이 "한 번도 안 박은 사람은
절대 안 잡힌다"의 보증이라, 이 값을 11 위로 올리면 완주가 기본이라는 원칙
자체가 깨진다.

이 값들이 만드는 시간표: 40초에 상한 도달(압박 전환점), 57.7초에 무사고 완주,
75.2초에 벽이 결승선 도달. 그 사이 17.5초가 실수 예산이고 스턴 0.8초로 치면
약 22번이다.

group을 비워 둬 클·서 양쪽 생성물에 다 들어간다 — 벽 위치는 서버가 잡을 때도,
클라가 그릴 때도 필요하다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SUnLXZFg9TeqE7mgvUt1Vp
</commit_message>
<xml_diff>
--- a/table/Datas/#FlappyConfig.xlsx
+++ b/table/Datas/#FlappyConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,26 @@
           <t>dash_charge_dive</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>chaser_start_x</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>chaser_initial_speed</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>chaser_acceleration</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>chaser_max_speed</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -569,6 +589,26 @@
           <t>float</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -651,6 +691,26 @@
       <c r="O4" t="inlineStr">
         <is>
           <t>dash_charge_dive</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>chaser_start_x</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>chaser_initial_speed</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>chaser_acceleration</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>chaser_max_speed</t>
         </is>
       </c>
     </row>
@@ -696,6 +756,18 @@
       </c>
       <c r="O5" t="n">
         <v>1.2</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-60</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>7</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="S5" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>